<commit_message>
Sync coPresentations move + updated Excel exports with current source metadata
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/exports/connect-the-dots-data.xlsx
+++ b/tools/exports/connect-the-dots-data.xlsx
@@ -40668,7 +40668,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>audhd</t>
+          <t>AuDHD</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -40703,7 +40703,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>fibro-mecfs</t>
+          <t>Fibromyalgia + ME/CFS</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -40738,7 +40738,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>depression-anxiety</t>
+          <t>Depression + Anxiety</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -41578,7 +41578,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>audhd</t>
+          <t>AuDHD</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -41613,7 +41613,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>hypermobility-pots-mcas</t>
+          <t>Hypermobility + POTS + MCAS</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -41648,7 +41648,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>fibro-mecfs</t>
+          <t>Fibromyalgia + ME/CFS</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -41683,7 +41683,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>depression-anxiety</t>
+          <t>Depression + Anxiety</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -42418,7 +42418,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>audhd</t>
+          <t>AuDHD</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -42453,7 +42453,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>hypermobility-pots-mcas</t>
+          <t>Hypermobility + POTS + MCAS</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -42488,7 +42488,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>fibro-mecfs</t>
+          <t>Fibromyalgia + ME/CFS</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -42523,7 +42523,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>depression-anxiety</t>
+          <t>Depression + Anxiety</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -43013,7 +43013,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>audhd</t>
+          <t>AuDHD</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -43048,7 +43048,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>hypermobility-pots-mcas</t>
+          <t>Hypermobility + POTS + MCAS</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
@@ -43083,7 +43083,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>fibro-mecfs</t>
+          <t>Fibromyalgia + ME/CFS</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -43118,7 +43118,7 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>depression-anxiety</t>
+          <t>Depression + Anxiety</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
@@ -43643,7 +43643,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>audhd</t>
+          <t>AuDHD</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
@@ -43678,7 +43678,7 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>hypermobility-pots-mcas</t>
+          <t>Hypermobility + POTS + MCAS</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -43713,7 +43713,7 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>fibro-mecfs</t>
+          <t>Fibromyalgia + ME/CFS</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
@@ -44063,7 +44063,7 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>audhd</t>
+          <t>AuDHD</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
@@ -44098,7 +44098,7 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>depression-anxiety</t>
+          <t>Depression + Anxiety</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
@@ -44483,7 +44483,7 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>audhd</t>
+          <t>AuDHD</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
@@ -44518,7 +44518,7 @@
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>atopic-triad</t>
+          <t>Atopic Triad</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
@@ -44903,7 +44903,7 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>audhd</t>
+          <t>AuDHD</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
@@ -45253,7 +45253,7 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>audhd</t>
+          <t>AuDHD</t>
         </is>
       </c>
       <c r="E157" t="inlineStr">
@@ -45603,7 +45603,7 @@
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>audhd</t>
+          <t>AuDHD</t>
         </is>
       </c>
       <c r="E167" t="inlineStr">
@@ -45638,7 +45638,7 @@
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>depression-anxiety</t>
+          <t>Depression + Anxiety</t>
         </is>
       </c>
       <c r="E168" t="inlineStr">
@@ -45988,7 +45988,7 @@
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>audhd</t>
+          <t>AuDHD</t>
         </is>
       </c>
       <c r="E178" t="inlineStr">
@@ -46023,7 +46023,7 @@
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>hypermobility-pots-mcas</t>
+          <t>Hypermobility + POTS + MCAS</t>
         </is>
       </c>
       <c r="E179" t="inlineStr">
@@ -46058,7 +46058,7 @@
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>depression-anxiety</t>
+          <t>Depression + Anxiety</t>
         </is>
       </c>
       <c r="E180" t="inlineStr">

</xml_diff>

<commit_message>
v1.4-beta — Sharing, deep links, structured data, dark mode fixes
</commit_message>
<xml_diff>
--- a/tools/exports/connect-the-dots-data.xlsx
+++ b/tools/exports/connect-the-dots-data.xlsx
@@ -23441,7 +23441,7 @@
         <v>0</v>
       </c>
       <c r="L356" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="357">
@@ -23588,7 +23588,7 @@
         <v>0</v>
       </c>
       <c r="L359" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="360">
@@ -23686,7 +23686,7 @@
         <v>0</v>
       </c>
       <c r="L361" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="362">
@@ -23735,7 +23735,7 @@
         <v>0</v>
       </c>
       <c r="L362" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="363">

</xml_diff>